<commit_message>
Add Xiangling's remap draft file
</commit_message>
<xml_diff>
--- a/Data/RemapDrafts/XianglingRemapDraft.xlsx
+++ b/Data/RemapDrafts/XianglingRemapDraft.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Computer\Games\Genshin\Repos\Repos\Fix-Raiden-Boss\Data\RemapDrafts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DB34FEA-ACC7-4826-9F76-7F6C38F99E2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62096884-EBB3-4646-96E3-1650EC397CF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="34620" windowHeight="13900" xr2:uid="{F8BD3DC3-F6C2-4809-8B31-A9D12C142664}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="V5.3 - Xiangling to Cheer" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'V5.3 - Xiangling to Cheer'!$A$1:$D$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'V5.3 - Xiangling to Cheer'!$A$1:$D$78</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1304,10 +1304,11 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D1" xr:uid="{0A8DBCD4-58C9-4D83-BA94-EBBD7745B45F}"/>
+  <autoFilter ref="A1:D78" xr:uid="{0A8DBCD4-58C9-4D83-BA94-EBBD7745B45F}"/>
   <conditionalFormatting sqref="B2:B78">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Xiangling's Vertex Group Remap Draft
</commit_message>
<xml_diff>
--- a/Data/RemapDrafts/XianglingRemapDraft.xlsx
+++ b/Data/RemapDrafts/XianglingRemapDraft.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Computer\Games\Genshin\Repos\Repos\Fix-Raiden-Boss\Data\RemapDrafts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D21633F7-01F5-4F04-9D8B-167772B42506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C3BD051-AF54-4DE2-88C0-89DA9EE323BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="34620" windowHeight="13900" activeTab="1" xr2:uid="{F8BD3DC3-F6C2-4809-8B31-A9D12C142664}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="34620" windowHeight="13900" xr2:uid="{F8BD3DC3-F6C2-4809-8B31-A9D12C142664}"/>
   </bookViews>
   <sheets>
     <sheet name="V5.3 - Xiangling to Cheer" sheetId="1" r:id="rId1"/>
@@ -2323,5 +2323,6 @@
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>